<commit_message>
Drop the group code from the team name and widen columns
Rename the team to "20/80" without the group suffix everywhere: the
stakeholder register, the grid footer, the RACI matrix, the communication
plan and both filled templates, including the project team directory and
the body text of the communications management plan.

Widen the columns of the register, the RACI activity column and the
communication plan so the wrapped text fits without clipping, and raise
the row heights to match.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BA/Part 1_Stakeholder Analysis amp Management-20260912/Artifacts/1. Stakeholder Register_VNS.xlsx
+++ b/BA/Part 1_Stakeholder Analysis amp Management-20260912/Artifacts/1. Stakeholder Register_VNS.xlsx
@@ -527,19 +527,19 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="56" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="70" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="2" ht="26" customHeight="1">
@@ -793,7 +793,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="62" customHeight="1">
+    <row r="12" ht="74" customHeight="1">
       <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Lviv Polytechnic National University</t>
@@ -860,7 +860,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="62" customHeight="1">
+    <row r="13" ht="74" customHeight="1">
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Ministry of Education and Science of Ukraine</t>
@@ -927,7 +927,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="62" customHeight="1">
+    <row r="14" ht="74" customHeight="1">
       <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Nataliia Shakhovska</t>
@@ -994,7 +994,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="62" customHeight="1">
+    <row r="15" ht="74" customHeight="1">
       <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Nataliia Boiko</t>
@@ -1061,7 +1061,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="62" customHeight="1">
+    <row r="16" ht="74" customHeight="1">
       <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Technical Department of Lviv Polytechnic</t>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="62" customHeight="1">
+    <row r="17" ht="74" customHeight="1">
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>End users — Lviv Polytechnic students</t>
@@ -1195,7 +1195,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="62" customHeight="1">
+    <row r="18" ht="74" customHeight="1">
       <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Kostiantyn Holovskyi</t>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Project team “20/80”, group SHI-2025</t>
+          <t>Project team “20/80”</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
@@ -1262,7 +1262,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="62" customHeight="1">
+    <row r="19" ht="74" customHeight="1">
       <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Nazar Zankovych</t>
@@ -1280,7 +1280,7 @@
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Project team “20/80”, group SHI-2025</t>
+          <t>Project team “20/80”</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
@@ -1329,7 +1329,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="62" customHeight="1">
+    <row r="20" ht="74" customHeight="1">
       <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Andrii Lysun</t>
@@ -1347,7 +1347,7 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Project team “20/80”, group SHI-2025</t>
+          <t>Project team “20/80”</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
@@ -1396,7 +1396,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="62" customHeight="1">
+    <row r="21" ht="74" customHeight="1">
       <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Denys Lunhul</t>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Project team “20/80”, group SHI-2025</t>
+          <t>Project team “20/80”</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
@@ -1463,7 +1463,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="62" customHeight="1">
+    <row r="22" ht="74" customHeight="1">
       <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Yaroslav Shevchuk</t>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Project team “20/80”, group SHI-2025</t>
+          <t>Project team “20/80”</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
@@ -1530,7 +1530,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="62" customHeight="1">
+    <row r="23" ht="74" customHeight="1">
       <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Volodymyr Kamelchuk</t>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Project team “20/80”, group SHI-2025</t>
+          <t>Project team “20/80”</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">

</xml_diff>